<commit_message>
Add swap-batch up/down counts, zero-sales revival, and gain concentration for full September
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/missacc_2027_growth_analysis/missacc_ed_image_swap_effect.xlsx
+++ b/missacc_2027_growth_analysis/missacc_ed_image_swap_effect.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="批次汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="SPU明细(430款)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="口径与结论" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="全月件数分布" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="批次汇总" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SPU明细(430款)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="口径与结论" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'SPU明细(430款)'!$A$1:$K$409</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SPU明细(430款)'!$A$1:$K$409</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%;0"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -59,9 +63,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,6 +439,610 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>口径</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>组别</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>两月在架</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>8月件数</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>9月件数</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>日均环比</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>变好款</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>变好占比</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>持平款</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>持平占比</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>变差款</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>变差占比</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>7月换图</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>112</v>
+      </c>
+      <c r="C4" t="n">
+        <v>521</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>618</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8月换图</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>147</v>
+      </c>
+      <c r="C5" t="n">
+        <v>330</v>
+      </c>
+      <c r="D5" t="n">
+        <v>512</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0.603</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.578</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.143</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5-6月换图</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>79</v>
+      </c>
+      <c r="C6" t="n">
+        <v>253</v>
+      </c>
+      <c r="D6" t="n">
+        <v>184</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>-0.248</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.797</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.152</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>未换图对照</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>375</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2168</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1879</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>-0.104</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>201</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.283</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9月上旬(不参与对照)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>37</v>
+      </c>
+      <c r="C8" t="n">
+        <v>108</v>
+      </c>
+      <c r="D8" t="n">
+        <v>127</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>8月零销款</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>8月零销款数</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>9月≥2件</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>复活率</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>9月仅1件</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>零销款9月合计件数</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9月人均件数</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>7月换图</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>38</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="E11" t="n">
+        <v>14</v>
+      </c>
+      <c r="F11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8月换图</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>60</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>16</v>
+      </c>
+      <c r="F12" t="n">
+        <v>36</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>5-6月换图</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>42</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>未换图对照</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>82</v>
+      </c>
+      <c r="C14" t="n">
+        <v>13</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="E14" t="n">
+        <v>27</v>
+      </c>
+      <c r="F14" t="n">
+        <v>63</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>净增量来自哪个起点（9月件数−8月件数）</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>8月0件</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>8月1-5件</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>8月6-15件</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>8月16件以上</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>7月换图</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" t="n">
+        <v>13</v>
+      </c>
+      <c r="D17" t="n">
+        <v>42</v>
+      </c>
+      <c r="E17" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8月换图</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>36</v>
+      </c>
+      <c r="C18" t="n">
+        <v>113</v>
+      </c>
+      <c r="D18" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>5-6月换图</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-21</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-10</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-46</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>未换图对照</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>63</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-25</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-116</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-211</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>正增量集中度</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>前10%款数</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>前10%占正增量</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>前5款占正增量</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>7月换图</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>11</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.398</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>前10%占净增量超过100%，是因为其余款有减量，净额被缩小</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>8月换图</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>15</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>0.597</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>对照的前10%占正增量也是63.5%，集中度不是换图特有的</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>未换图对照</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>38</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0.188</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -655,8 +1271,6 @@
           <t>净效应</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -679,8 +1293,6 @@
       <c r="F9" t="n">
         <v>1.43</v>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -703,8 +1315,6 @@
       <c r="F10" t="n">
         <v>1.52</v>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -727,8 +1337,6 @@
       <c r="F11" t="n">
         <v>0.24</v>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -751,8 +1359,6 @@
       <c r="F12" t="n">
         <v>1.01</v>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -781,15 +1387,13 @@
           <t>27倍</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21242,7 +21846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Count a first sale of a zero-sales SKU as revival, and split out 1-unit cases
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/missacc_2027_growth_analysis/missacc_ed_image_swap_effect.xlsx
+++ b/missacc_2027_growth_analysis/missacc_ed_image_swap_effect.xlsx
@@ -458,7 +458,7 @@
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>口径</t>
+          <t>口径：两月都在架的 ED。变好 = 9月件数−8月件数 ≥2；变差 = 8月−9月 ≥2；差 0 或 1 件为持平。零销款复活 = 8月 0 件且 9月 ≥1 件（1 件与 ≥2 件分开计，卖出 1 件即算进步）。对照 = 未换图、上架早于 2026-01。9月上旬批次换完不满一个月，不与对照比较。</t>
         </is>
       </c>
     </row>
@@ -710,135 +710,152 @@
           <t>8月零销款</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>8月零销款数</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>9月仍为0</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>9月1件</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>9月≥2件</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>复活（≥1件）</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>复活率</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>9月仅1件</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>零销款9月合计件数</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>9月人均件数</t>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>9月合计件数</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>7月换图</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="3" t="n">
-        <v>0.105</v>
-      </c>
-      <c r="E11" t="n">
-        <v>14</v>
-      </c>
-      <c r="F11" t="n">
+      <c r="F11" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0.4736842105263158</v>
+      </c>
+      <c r="H11" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="G11" s="6" t="n">
-        <v>0.66</v>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>8月换图</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D12" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>16</v>
-      </c>
-      <c r="F12" t="n">
+      <c r="F12" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.3666666666666666</v>
+      </c>
+      <c r="H12" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="G12" s="6" t="n">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>5-6月换图</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
+      <c r="C13" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="D13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="F13" t="n">
+      <c r="E13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="G13" s="6" t="n">
-        <v>0.19</v>
+      <c r="G13" s="3" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>未换图对照</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="7" t="n">
         <v>82</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="E14" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="D14" s="3" t="n">
-        <v>0.159</v>
-      </c>
-      <c r="E14" t="n">
-        <v>27</v>
-      </c>
-      <c r="F14" t="n">
+      <c r="F14" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.4878048780487805</v>
+      </c>
+      <c r="H14" s="7" t="n">
         <v>63</v>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>0.77</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Attribute batch net gains to the few SKUs with large unit increases
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/missacc_2027_growth_analysis/missacc_ed_image_swap_effect.xlsx
+++ b/missacc_2027_growth_analysis/missacc_ed_image_swap_effect.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1044,6 +1044,93 @@
       </c>
       <c r="D25" s="3" t="n">
         <v>0.188</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>批次净增量来源</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>涨≥10件的款数</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>这些款的增量</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>占该批净增量</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>7月换图</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" t="n">
+        <v>96</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>0.9896907216494846</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>等于净增量+97的全部；其余款加减相抵</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>8月换图</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" t="n">
+        <v>105</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>0.5769230769230769</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>占净增量+182的58%；涨≥5件的19款盖住全部净增量</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>5-6月换图</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>没有任何一款涨满5件，整批净-69</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>